<commit_message>
Q3 Digital Engagement & Product Holdings sql data added  in excel
</commit_message>
<xml_diff>
--- a/Q1_Q2_Q3_SQL_Analysis/Q3_digital_engagement_product_holdings/Q3_digital_engagement_product_holdings.xlsx
+++ b/Q1_Q2_Q3_SQL_Analysis/Q3_digital_engagement_product_holdings/Q3_digital_engagement_product_holdings.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mine\Dialog\dialog-finance-analytics\Q1_Q2_Q3_SQL_Analysis\Q3_digital_engagement_product_holdings\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097D3936-79A5-43A0-83F0-F21B1B767E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Q3_digital_engagement_produc" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +24,131 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
+  <si>
+    <t>Q3: Digital Engagement &amp; Product Holdings</t>
+  </si>
+  <si>
+    <t>mobile_app_user</t>
+  </si>
+  <si>
+    <t>customer_count</t>
+  </si>
+  <si>
+    <t>avg_savings_balance</t>
+  </si>
+  <si>
+    <t>median_savings_balance</t>
+  </si>
+  <si>
+    <t>total_savings</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Q3a — Do mobile app users maintain higher savings balances?</t>
+  </si>
+  <si>
+    <t>Q3b — Cross-sell opportunity</t>
+  </si>
+  <si>
+    <t>cross_sell_customer_count</t>
+  </si>
+  <si>
+    <t>total_savings_held_lkr</t>
+  </si>
+  <si>
+    <t>avg_savings_per_customer</t>
+  </si>
+  <si>
+    <t>Breakdown by Segment (to prioritise who to target first)</t>
+  </si>
+  <si>
+    <t>customer_segment</t>
+  </si>
+  <si>
+    <t>cross_sell_customers</t>
+  </si>
+  <si>
+    <t>total_savings_lkr</t>
+  </si>
+  <si>
+    <t>avg_savings</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>Regular</t>
+  </si>
+  <si>
+    <t>Starter</t>
+  </si>
+  <si>
+    <t>Breakdown by Acquisition Channel (to target via the right channel)</t>
+  </si>
+  <si>
+    <t>acquisition_channel</t>
+  </si>
+  <si>
+    <t>Branch</t>
+  </si>
+  <si>
+    <t>Digital</t>
+  </si>
+  <si>
+    <t>Referral</t>
+  </si>
+  <si>
+    <t>Agent</t>
+  </si>
+  <si>
+    <t>Q3c — Best Acquisition Channel: highest savings + lowest default</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Step 1: Average savings by channel</t>
+  </si>
+  <si>
+    <t>total_customers</t>
+  </si>
+  <si>
+    <t>Step 2: Default rate by channel</t>
+  </si>
+  <si>
+    <t>loan_customers</t>
+  </si>
+  <si>
+    <t>defaulted</t>
+  </si>
+  <si>
+    <t> Step 3: Combined view — savings and default side by side</t>
+  </si>
+  <si>
+    <t>defaulted_loans</t>
+  </si>
+  <si>
+    <t>total_loans</t>
+  </si>
+  <si>
+    <t>default_rate_pct %</t>
+  </si>
+  <si>
+    <t>default_rate_pct  %</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +156,49 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,14 +213,62 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="11">
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="\L\K\R\ #,##0.00"/>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{5A49A66A-2EFE-46D0-9F38-EB125D8EA2A3}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -66,6 +278,98 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6FBBCF73-8A7F-4BF1-B480-AA636AACBBC1}" name="Table1" displayName="Table1" ref="B8:F10" totalsRowShown="0">
+  <autoFilter ref="B8:F10" xr:uid="{6FBBCF73-8A7F-4BF1-B480-AA636AACBBC1}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{B7AA0A14-C0D4-43C9-9167-A40D9D6EABDC}" name="mobile_app_user"/>
+    <tableColumn id="2" xr3:uid="{6C69326C-D622-4C5F-999C-5C84B2C687F3}" name="customer_count"/>
+    <tableColumn id="3" xr3:uid="{DD4C349E-64E1-4AA2-A578-056846376E01}" name="avg_savings_balance" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{203CD9BF-F91C-4CEC-BA6D-1D64FFA53D98}" name="median_savings_balance" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{0D053410-057F-431F-8D33-94009A861476}" name="total_savings" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8B6D093E-A11E-487F-8DB6-631D01C32788}" name="Table2" displayName="Table2" ref="B16:D17" totalsRowShown="0">
+  <autoFilter ref="B16:D17" xr:uid="{8B6D093E-A11E-487F-8DB6-631D01C32788}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{DCD0CF8C-9351-4FAA-AFB8-A05A753BDF10}" name="cross_sell_customer_count"/>
+    <tableColumn id="2" xr3:uid="{24F6D4D0-D14D-4A4C-9201-A039DEA67A18}" name="total_savings_held_lkr" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{BD5C5A38-0AD8-4B00-99FB-54A9FCEE8BDB}" name="avg_savings_per_customer" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BD581072-CAD1-4C9D-A060-1A26352E22F7}" name="Table3" displayName="Table3" ref="B23:E26" totalsRowShown="0">
+  <autoFilter ref="B23:E26" xr:uid="{BD581072-CAD1-4C9D-A060-1A26352E22F7}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{40D9D2E7-FA85-41D9-8188-D5C0FA85CDDD}" name="customer_segment"/>
+    <tableColumn id="2" xr3:uid="{A62730FE-1C47-41F1-8C30-AFD2B1777E03}" name="cross_sell_customers"/>
+    <tableColumn id="3" xr3:uid="{27A9798B-AD6B-4C65-AAD7-2236AD17278D}" name="total_savings_lkr" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{758BA49A-9E92-4C97-8917-CAB7DD8A8BD4}" name="avg_savings" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B9DC4926-1A64-4275-9065-B1BC7D2E4CFC}" name="Table4" displayName="Table4" ref="B32:E36" totalsRowShown="0">
+  <autoFilter ref="B32:E36" xr:uid="{B9DC4926-1A64-4275-9065-B1BC7D2E4CFC}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{91227D68-C0D2-41B9-8B0D-B1AF44736916}" name="acquisition_channel"/>
+    <tableColumn id="2" xr3:uid="{F995CCF1-8B9A-4F6E-92E8-4F27CF4A5E7C}" name="cross_sell_customers"/>
+    <tableColumn id="3" xr3:uid="{CD4AFB79-5443-4B39-B140-977F1F395FFD}" name="total_savings_lkr" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{19111F9E-01FC-41FB-9678-82DB7CC01A16}" name="avg_savings" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CA361C53-FF89-43CA-AFD4-E35B443AF73E}" name="Table5" displayName="Table5" ref="B44:D48" totalsRowShown="0">
+  <autoFilter ref="B44:D48" xr:uid="{CA361C53-FF89-43CA-AFD4-E35B443AF73E}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{EA9762E7-587E-481C-B80B-981D058F5D83}" name="acquisition_channel"/>
+    <tableColumn id="2" xr3:uid="{AC1F78F5-50D4-48B2-AD80-A89B209EF93F}" name="total_customers"/>
+    <tableColumn id="3" xr3:uid="{FF1E1F82-BE78-44A5-9C44-A1A45659BE00}" name="avg_savings_balance" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5E335209-DF19-454A-AD90-8DBD479FEAB0}" name="Table6" displayName="Table6" ref="B54:E58" totalsRowShown="0">
+  <autoFilter ref="B54:E58" xr:uid="{5E335209-DF19-454A-AD90-8DBD479FEAB0}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{ABF8F9F5-5DEE-45A3-91F4-5EB8F1AE9708}" name="acquisition_channel"/>
+    <tableColumn id="2" xr3:uid="{66A64835-D927-433A-858B-94A11F53D2EA}" name="loan_customers"/>
+    <tableColumn id="3" xr3:uid="{EA7E6B62-EA8D-4CD5-9DB5-173C5841BC11}" name="defaulted"/>
+    <tableColumn id="4" xr3:uid="{ACF9B6BD-75CF-41F9-BE7F-7242C4E92B94}" name="default_rate_pct  %"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{312BC90E-AA3A-4C22-B410-0A21DD21842E}" name="Table7" displayName="Table7" ref="B64:G68" totalsRowShown="0">
+  <autoFilter ref="B64:G68" xr:uid="{312BC90E-AA3A-4C22-B410-0A21DD21842E}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{E613C8D8-93E7-46D8-9B3B-1565E3ABCFA4}" name="acquisition_channel"/>
+    <tableColumn id="2" xr3:uid="{6F1EFE9F-6892-4FD5-B2DF-F0EC67BB2705}" name="total_customers"/>
+    <tableColumn id="3" xr3:uid="{47511CE3-E202-46BE-81EC-887971DE28BF}" name="avg_savings" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{EC2E2EDB-4505-4DC3-A25F-647152940E25}" name="defaulted_loans"/>
+    <tableColumn id="5" xr3:uid="{E3F05355-5DDE-4B11-8E51-BA2C84D4486E}" name="total_loans"/>
+    <tableColumn id="6" xr3:uid="{93A0FE08-DD2D-46B2-AB6F-5DA8CEE0B9DB}" name="default_rate_pct %"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +634,521 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B3:G68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="6" spans="2:6" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9">
+        <v>164</v>
+      </c>
+      <c r="D9" s="6">
+        <v>798127.91</v>
+      </c>
+      <c r="E9" s="6">
+        <v>444521.96</v>
+      </c>
+      <c r="F9" s="6">
+        <v>130892977.86</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10">
+        <v>325</v>
+      </c>
+      <c r="D10" s="6">
+        <v>761403.81</v>
+      </c>
+      <c r="E10" s="6">
+        <v>448866.68</v>
+      </c>
+      <c r="F10" s="6">
+        <v>247456238.93000001</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>251</v>
+      </c>
+      <c r="C17" s="6">
+        <v>222385271.58000001</v>
+      </c>
+      <c r="D17" s="6">
+        <v>885997.1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B21" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24">
+        <v>57</v>
+      </c>
+      <c r="D24" s="6">
+        <v>152252879.34999999</v>
+      </c>
+      <c r="E24" s="6">
+        <v>2671103.15</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25">
+        <v>146</v>
+      </c>
+      <c r="D25" s="6">
+        <v>64491752.689999998</v>
+      </c>
+      <c r="E25" s="6">
+        <v>441724.33</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26">
+        <v>45</v>
+      </c>
+      <c r="D26" s="6">
+        <v>3954785.03</v>
+      </c>
+      <c r="E26" s="6">
+        <v>87884.11</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B30" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>23</v>
+      </c>
+      <c r="C33">
+        <v>64</v>
+      </c>
+      <c r="D33" s="6">
+        <v>68037948.099999994</v>
+      </c>
+      <c r="E33" s="6">
+        <v>1063092.94</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34">
+        <v>67</v>
+      </c>
+      <c r="D34" s="6">
+        <v>58227847.920000002</v>
+      </c>
+      <c r="E34" s="6">
+        <v>869072.36</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35">
+        <v>62</v>
+      </c>
+      <c r="D35" s="6">
+        <v>55943173.359999999</v>
+      </c>
+      <c r="E35" s="6">
+        <v>902309.25</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36">
+        <v>58</v>
+      </c>
+      <c r="D36" s="6">
+        <v>40176302.200000003</v>
+      </c>
+      <c r="E36" s="6">
+        <v>692694.87</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="B40" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B41" s="1"/>
+    </row>
+    <row r="42" spans="2:5" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B42" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>22</v>
+      </c>
+      <c r="C44" t="s">
+        <v>29</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>23</v>
+      </c>
+      <c r="C45">
+        <v>118</v>
+      </c>
+      <c r="D45" s="6">
+        <v>841984.38</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>24</v>
+      </c>
+      <c r="C46">
+        <v>129</v>
+      </c>
+      <c r="D46" s="6">
+        <v>830903.09</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>25</v>
+      </c>
+      <c r="C47">
+        <v>126</v>
+      </c>
+      <c r="D47" s="6">
+        <v>768937.97</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>26</v>
+      </c>
+      <c r="C48">
+        <v>116</v>
+      </c>
+      <c r="D48" s="6">
+        <v>645882.56000000006</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B52" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52" s="2"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>22</v>
+      </c>
+      <c r="C54" t="s">
+        <v>31</v>
+      </c>
+      <c r="D54" t="s">
+        <v>32</v>
+      </c>
+      <c r="E54" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>26</v>
+      </c>
+      <c r="C55">
+        <v>56</v>
+      </c>
+      <c r="D55">
+        <v>3</v>
+      </c>
+      <c r="E55">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>24</v>
+      </c>
+      <c r="C56">
+        <v>54</v>
+      </c>
+      <c r="D56">
+        <v>6</v>
+      </c>
+      <c r="E56">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>23</v>
+      </c>
+      <c r="C57">
+        <v>51</v>
+      </c>
+      <c r="D57">
+        <v>6</v>
+      </c>
+      <c r="E57">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>25</v>
+      </c>
+      <c r="C58">
+        <v>55</v>
+      </c>
+      <c r="D58">
+        <v>7</v>
+      </c>
+      <c r="E58">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B62" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>22</v>
+      </c>
+      <c r="C64" t="s">
+        <v>29</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E64" t="s">
+        <v>34</v>
+      </c>
+      <c r="F64" t="s">
+        <v>35</v>
+      </c>
+      <c r="G64" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>23</v>
+      </c>
+      <c r="C65">
+        <v>123</v>
+      </c>
+      <c r="D65" s="6">
+        <v>841984.38</v>
+      </c>
+      <c r="E65">
+        <v>6</v>
+      </c>
+      <c r="F65">
+        <v>51</v>
+      </c>
+      <c r="G65">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>24</v>
+      </c>
+      <c r="C66">
+        <v>131</v>
+      </c>
+      <c r="D66" s="6">
+        <v>830903.09</v>
+      </c>
+      <c r="E66">
+        <v>6</v>
+      </c>
+      <c r="F66">
+        <v>54</v>
+      </c>
+      <c r="G66">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>25</v>
+      </c>
+      <c r="C67">
+        <v>129</v>
+      </c>
+      <c r="D67" s="6">
+        <v>768937.97</v>
+      </c>
+      <c r="E67">
+        <v>7</v>
+      </c>
+      <c r="F67">
+        <v>57</v>
+      </c>
+      <c r="G67">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>26</v>
+      </c>
+      <c r="C68">
+        <v>117</v>
+      </c>
+      <c r="D68" s="6">
+        <v>645882.56000000006</v>
+      </c>
+      <c r="E68">
+        <v>3</v>
+      </c>
+      <c r="F68">
+        <v>56</v>
+      </c>
+      <c r="G68">
+        <v>5.4</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="7">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>